<commit_message>
Created groundwater head contours (didn't push folder because some gis files were too big).  Calculated lake precipitation and added to .lak file.  Double-checked that streamflow in the tab files is correct.  Double-checked that we're adjusting the right parameters.
</commit_message>
<xml_diff>
--- a/gsflow/pilot_points_near_gw_wells.xlsx
+++ b/gsflow/pilot_points_near_gw_wells.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="21">
   <si>
     <t>gw well</t>
   </si>
@@ -69,6 +69,24 @@
   </si>
   <si>
     <t>v6</t>
+  </si>
+  <si>
+    <t>measured &gt; modelled ?</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>nearby pilot point K values need to increase/decrease</t>
+  </si>
+  <si>
+    <t>increase</t>
+  </si>
+  <si>
+    <t>decrease</t>
   </si>
 </sst>
 </file>
@@ -386,21 +404,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="49.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -408,165 +428,249 @@
       <c r="E1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2">
         <v>10</v>
       </c>
-      <c r="C2">
+      <c r="E2">
         <v>42</v>
       </c>
-      <c r="D2">
+      <c r="F2">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5">
         <v>7</v>
       </c>
-      <c r="C5">
+      <c r="E5">
         <v>36</v>
       </c>
-      <c r="D5">
+      <c r="F5">
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6">
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6">
         <v>6</v>
       </c>
-      <c r="C6">
+      <c r="E6">
         <v>35</v>
       </c>
-      <c r="D6">
+      <c r="F6">
         <v>25</v>
       </c>
-      <c r="E6">
+      <c r="G6">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7">
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7">
         <v>5</v>
       </c>
-      <c r="C7">
+      <c r="E7">
         <v>12</v>
       </c>
-      <c r="D7">
+      <c r="F7">
         <v>21</v>
       </c>
-      <c r="E7">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G7">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8">
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8">
         <v>3</v>
       </c>
-      <c r="C8">
-        <v>16</v>
-      </c>
-      <c r="D8">
+      <c r="E8">
+        <v>16</v>
+      </c>
+      <c r="F8">
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
-      <c r="B9">
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
-      <c r="B10">
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="B11">
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11">
         <v>1</v>
       </c>
-      <c r="C11">
+      <c r="E11">
         <v>14</v>
       </c>
-      <c r="D11">
+      <c r="F11">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12">
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12">
         <v>13</v>
       </c>
-      <c r="C12">
+      <c r="E12">
         <v>47</v>
       </c>
-      <c r="D12">
+      <c r="F12">
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B13">
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13">
         <v>12</v>
       </c>
-      <c r="C13">
+      <c r="E13">
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14">
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14">
         <v>11</v>
       </c>
-      <c r="C14">
+      <c r="E14">
         <v>44</v>
       </c>
-      <c r="D14">
+      <c r="F14">
         <v>45</v>
       </c>
     </row>

</xml_diff>